<commit_message>
Ya casi, falta terminar la presentación
</commit_message>
<xml_diff>
--- a/outputs/Comparación_Ubicuidad.xlsx
+++ b/outputs/Comparación_Ubicuidad.xlsx
@@ -17,10 +17,10 @@
     <t xml:space="preserve">Genérico</t>
   </si>
   <si>
-    <t xml:space="preserve">MySd</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Indice</t>
+    <t xml:space="preserve">Op1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Op2</t>
   </si>
   <si>
     <t xml:space="preserve">002 Botanas elaboradas con cereales</t>

</xml_diff>